<commit_message>
update dc measure secureCRT DTMX
</commit_message>
<xml_diff>
--- a/MsPFM/AIC8822/MsTables/20250108/WF_MEASURE_TABLE_20250108_1903.xlsx
+++ b/MsPFM/AIC8822/MsTables/20250108/WF_MEASURE_TABLE_20250108_1903.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="39">
   <si>
     <t>BOARD_NO</t>
   </si>
@@ -64,7 +64,7 @@
     <t>R_MASK_MAX</t>
   </si>
   <si>
-    <t>#A2</t>
+    <t>#A3</t>
   </si>
   <si>
     <t>ANT0</t>
@@ -76,30 +76,30 @@
     <t>RF1.8</t>
   </si>
   <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>7,42,58,106,122,138,155</t>
+  </si>
+  <si>
+    <t>5 11</t>
+  </si>
+  <si>
+    <t>0 0</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>r 403422c8</t>
+  </si>
+  <si>
     <t>Y</t>
   </si>
   <si>
-    <t>7,42,58,106,122,138,155</t>
-  </si>
-  <si>
-    <t>5 11</t>
-  </si>
-  <si>
-    <t>0 0</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>r 403422c8</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>testmode22_2024_1210_1040.bin</t>
+  </si>
+  <si>
+    <t>testmode22_dbg_tmx_vh_vbit_2003.bin</t>
   </si>
 </sst>
 </file>
@@ -1101,7 +1104,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
@@ -1201,19 +1204,19 @@
         <v>26</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1251,19 +1254,19 @@
         <v>26</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -1301,19 +1304,19 @@
         <v>26</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1351,19 +1354,19 @@
         <v>26</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P5" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1401,19 +1404,19 @@
         <v>26</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P6" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1451,19 +1454,19 @@
         <v>26</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1480,7 +1483,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>21</v>
@@ -1501,19 +1504,19 @@
         <v>26</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1530,7 +1533,7 @@
         <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>28</v>
@@ -1551,19 +1554,19 @@
         <v>26</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P9" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1580,7 +1583,7 @@
         <v>19</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>28</v>
@@ -1601,19 +1604,19 @@
         <v>26</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -1630,7 +1633,7 @@
         <v>36</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>21</v>
@@ -1651,19 +1654,19 @@
         <v>26</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -1680,7 +1683,7 @@
         <v>36</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>28</v>
@@ -1701,19 +1704,19 @@
         <v>26</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -1730,7 +1733,7 @@
         <v>36</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>28</v>
@@ -1751,84 +1754,320 @@
         <v>26</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="P13" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
+    <row r="14" spans="1:16">
+      <c r="A14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
+    <row r="15" spans="1:16">
+      <c r="A15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+    <row r="16" spans="1:16">
+      <c r="A16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P16" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="17" spans="1:15">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+    <row r="17" spans="1:16">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
+      <c r="A19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P19" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>